<commit_message>
fix: :bug: restablishing original settins for inc deployment
</commit_message>
<xml_diff>
--- a/backend/Creación de Ficha de Producto 3D.xlsx
+++ b/backend/Creación de Ficha de Producto 3D.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\dnthdev\proyectos\blackMichiEstudiov2\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4F8BD33-C424-4D83-A343-1FF1E8DD22DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07FF2DC5-873D-4A68-A139-A718B4395EF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="3105" windowWidth="17520" windowHeight="12480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Creación de Ficha de Producto 3" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: :sparkles: adding new products in excel
</commit_message>
<xml_diff>
--- a/backend/Creación de Ficha de Producto 3D.xlsx
+++ b/backend/Creación de Ficha de Producto 3D.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\dnthdev\proyectos\blackMichiEstudiov2\backend\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\dnthdev\proyectos\blackMichiEstudioPreProd\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07FF2DC5-873D-4A68-A139-A718B4395EF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBC7E53D-1C6B-4130-B33C-7C6807239503}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="3105" windowWidth="17520" windowHeight="12480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Creación de Ficha de Producto 3" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="103">
   <si>
     <t>SKU / ID</t>
   </si>
@@ -146,6 +146,189 @@
   </si>
   <si>
     <t>18 - 24 horas</t>
+  </si>
+  <si>
+    <t>BM-MIN-TNT-01</t>
+  </si>
+  <si>
+    <t>Macetero/Organizador Bloque TNT</t>
+  </si>
+  <si>
+    <t>Decoración / Gamer</t>
+  </si>
+  <si>
+    <t>Organizador cúbico con diseño de bloque TNT de Minecraft, impreso en piezas de colores.</t>
+  </si>
+  <si>
+    <t>Cubo funcional multiuso ideal para lápices o plantas pequeñas. Diseño geométrico fiel al videojuego con letras en relieve.</t>
+  </si>
+  <si>
+    <t>12 - 18 horas</t>
+  </si>
+  <si>
+    <t>Filamento PLA Rojo, Blanco y Negro. Ensamblado de alta precisión.</t>
+  </si>
+  <si>
+    <t>BM-EGI-ISI-01</t>
+  </si>
+  <si>
+    <t>Diosa Isis Alada - Edición Bronce</t>
+  </si>
+  <si>
+    <t>Figura detallada de la diosa Isis con alas extendidas sobre base jeroglífica.</t>
+  </si>
+  <si>
+    <t>Representación de la maternidad y el nacimiento. Impresión de alta definición con acabado sedoso que resalta el plumaje.</t>
+  </si>
+  <si>
+    <t>Filamento PLA Silk Bronce / Dorado de alta calidad.</t>
+  </si>
+  <si>
+    <t>BM-GEO-EST-01</t>
+  </si>
+  <si>
+    <t>Estructura Geométrica Estrellada</t>
+  </si>
+  <si>
+    <t>Decoración / Minimalista</t>
+  </si>
+  <si>
+    <t>Figura de geometría sagrada con estructura de poliedro estrellado calado.</t>
+  </si>
+  <si>
+    <t>Pieza decorativa abstracta de gran complejidad visual. Estructura ligera pero resistente con diseño de líneas limpias.</t>
+  </si>
+  <si>
+    <t>10 - 15 horas</t>
+  </si>
+  <si>
+    <t>Filamento PLA Amarillo Mate / Fluor.</t>
+  </si>
+  <si>
+    <t>BM-GEO-FLO-01</t>
+  </si>
+  <si>
+    <t>Mandala "Flor de la Vida"</t>
+  </si>
+  <si>
+    <t>Decoración / Pared</t>
+  </si>
+  <si>
+    <t>Panel decorativo circular con el símbolo de la Flor de la Vida en relieve.</t>
+  </si>
+  <si>
+    <t>Arte mural geométrico que simboliza la creación. Diseño simétrico perfecto para armonización de espacios.</t>
+  </si>
+  <si>
+    <t>Filamento PLA Plata / Gris Metalizado.</t>
+  </si>
+  <si>
+    <t>BM-EGI-SEC-01</t>
+  </si>
+  <si>
+    <t>Estatua Diosa Sekhmet - Efecto Granito</t>
+  </si>
+  <si>
+    <t>Escultura de la diosa Sekhmet con cabeza de leona y disco solar.</t>
+  </si>
+  <si>
+    <t>Réplica con textura de piedra natural. Representa la fuerza y el poder. Acabado post-procesado para simular roca antigua.</t>
+  </si>
+  <si>
+    <t>24 - 30 horas</t>
+  </si>
+  <si>
+    <t>Filamento PLA texturizado o pintado con efecto granito/piedra.</t>
+  </si>
+  <si>
+    <t>BM-ORG-MIN-01</t>
+  </si>
+  <si>
+    <t>Set de Mini Maceteros Orgánicos (3 unidades)</t>
+  </si>
+  <si>
+    <t>Decoración / Hogar</t>
+  </si>
+  <si>
+    <t>Trío de maceteros pequeños con texturas geométricas y orgánicas variables.</t>
+  </si>
+  <si>
+    <t>Set de 3 piezas blancas con diseños de espiral, polígonos y ondas. Ideales para suculentas o cactus de interior.</t>
+  </si>
+  <si>
+    <t>Filamento PLA Blanco Premium, acabado satinado.</t>
+  </si>
+  <si>
+    <t>BM-MIN-CRE-01</t>
+  </si>
+  <si>
+    <t>Macetero/Organizador Bloque Creeper</t>
+  </si>
+  <si>
+    <t>Organizador cúbico con el rostro icónico de un Creeper de Minecraft.</t>
+  </si>
+  <si>
+    <t>Cubo decorativo con insertos negros para profundidad visual. Perfecto para escritorios temáticos.</t>
+  </si>
+  <si>
+    <t>Filamento PLA Verde Lima y Negro.</t>
+  </si>
+  <si>
+    <t>BM-SW-RAZ-01</t>
+  </si>
+  <si>
+    <t>Nave Razor Crest - Modelo Coleccionista</t>
+  </si>
+  <si>
+    <t>Coleccionables / Star Wars</t>
+  </si>
+  <si>
+    <t>Réplica detallada de la nave Razor Crest de "The Mandalorian" en alta resolución.</t>
+  </si>
+  <si>
+    <t>Modelo a escala con gran detalle en motores, cañones y cabina. Ideal para entusiastas de la saga y modelismo.</t>
+  </si>
+  <si>
+    <t>36 - 48 horas</t>
+  </si>
+  <si>
+    <t>Filamento PLA Gris Espacial / Plata, post-procesado con lavado de sombras.</t>
+  </si>
+  <si>
+    <t>BM-CAT-WED-01</t>
+  </si>
+  <si>
+    <t>Pareja de Gatos de Boda - Novios</t>
+  </si>
+  <si>
+    <t>Decoración / Regalos</t>
+  </si>
+  <si>
+    <t>Figuras de pareja de gatos vestidos de novios con detalles pintados a mano.</t>
+  </si>
+  <si>
+    <t>Set romántico: gato negro con frac y gato blanco con ramo de flores. Ideal para toppers de torta o regalo de aniversario.</t>
+  </si>
+  <si>
+    <t>24 - 36 horas</t>
+  </si>
+  <si>
+    <t>Filamento PLA, Pintura Acrílica (Negro, Blanco, Azul, Rosa), Barniz protector.</t>
+  </si>
+  <si>
+    <t>BM-MIN-STE-01</t>
+  </si>
+  <si>
+    <t>Macetero/Organizador Bloque Steve</t>
+  </si>
+  <si>
+    <t>Organizador cúbico con el diseño del rostro de Steve de Minecraft.</t>
+  </si>
+  <si>
+    <t>Construcción multi-pieza para lograr los colores de piel, cabello y ojos sin pintura. Muy resistente.</t>
+  </si>
+  <si>
+    <t>Filamento PLA Marrón, Piel, Azul y Blanco.</t>
   </si>
 </sst>
 </file>
@@ -232,12 +415,6 @@
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -250,6 +427,12 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -486,214 +669,451 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
     </row>
     <row r="2" spans="1:10" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="10">
+      <c r="D2" s="8">
         <v>35000</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
     </row>
     <row r="3" spans="1:10" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="8">
         <v>45000</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
     </row>
     <row r="4" spans="1:10" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="8">
         <v>25000</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
     </row>
     <row r="5" spans="1:10" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="8">
         <v>55000</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
     </row>
     <row r="6" spans="1:10" ht="39" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="8">
         <v>60000</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-    </row>
-    <row r="7" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-    </row>
-    <row r="8" spans="1:10" ht="12.75" x14ac:dyDescent="0.2"/>
-    <row r="9" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-    </row>
-    <row r="10" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A10" s="1"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+    </row>
+    <row r="7" spans="1:10" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A7" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="10">
+        <v>15000</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A8" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" s="10">
+        <v>45000</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A9" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="10">
+        <v>12000</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A10" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="10">
+        <v>18000</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="11" spans="1:10" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="1"/>
-      <c r="B11" s="3"/>
-    </row>
-    <row r="12" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="1"/>
-      <c r="B12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="1"/>
+      <c r="A11" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="10">
+        <v>55000</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="10">
+        <v>20000</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="10">
+        <v>15000</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="D14" s="10">
+        <v>60000</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D15" s="10">
+        <v>35000</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="10">
+        <v>18000</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
-      <c r="B20" s="6"/>
+      <c r="B20" s="4"/>
     </row>
     <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
-      <c r="B21" s="6"/>
+      <c r="B21" s="4"/>
     </row>
     <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
-      <c r="B22" s="6"/>
+      <c r="B22" s="4"/>
     </row>
     <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="5"/>
-      <c r="B23" s="6"/>
+      <c r="A23" s="3"/>
+      <c r="B23" s="4"/>
     </row>
     <row r="27" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="4"/>
+      <c r="B27" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>